<commit_message>
Major Update to Pull/Clean Scripts
</commit_message>
<xml_diff>
--- a/Data_Raw/aa-screen-libraries.xlsx
+++ b/Data_Raw/aa-screen-libraries.xlsx
@@ -1,26 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\qman0\OneDrive\Desktop\Tiny Earth Project\Excel Sheets\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_B1AB8A2E0B4172F9F79504ADCEC60468250D9F79" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
   </bookViews>
   <sheets>
-    <sheet name="Table1" sheetId="1" r:id="rId1"/>
+    <sheet name="Table1" sheetId="1" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <definedNames/>
+  <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4246" uniqueCount="294">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="294">
   <si>
     <t>id</t>
   </si>
@@ -907,9 +902,14 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
@@ -937,21 +937,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <tableStyles defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotTableStyle1"/>
 </styleSheet>
 </file>
 
@@ -1275,19 +1267,24 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xml:space="preserve" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
   <dimension ref="A1:S452"/>
-  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="2" max="4" width="18.296875" customWidth="1"/>
-    <col min="6" max="6" width="18.296875" customWidth="1"/>
-    <col min="9" max="9" width="18.296875" customWidth="1"/>
-    <col min="14" max="14" width="18.296875" customWidth="1"/>
-    <col min="17" max="17" width="18.296875" customWidth="1"/>
-    <col min="19" max="19" width="18.296875" customWidth="1"/>
+    <col min="2" max="2" width="18.33203125" customWidth="true" style="0"/>
+    <col min="3" max="3" width="18.33203125" customWidth="true" style="0"/>
+    <col min="4" max="4" width="18.33203125" customWidth="true" style="0"/>
+    <col min="6" max="6" width="18.33203125" customWidth="true" style="0"/>
+    <col min="9" max="9" width="18.33203125" customWidth="true" style="0"/>
+    <col min="14" max="14" width="18.33203125" customWidth="true" style="0"/>
+    <col min="17" max="17" width="18.33203125" customWidth="true" style="0"/>
+    <col min="19" max="19" width="18.33203125" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:19">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1346,7 +1343,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:19">
       <c r="A2">
         <v>1014686</v>
       </c>
@@ -1405,7 +1402,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:19">
       <c r="A3">
         <v>1014691</v>
       </c>
@@ -1464,7 +1461,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:19">
       <c r="A4">
         <v>1014976</v>
       </c>
@@ -1523,7 +1520,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:19">
       <c r="A5">
         <v>1015050</v>
       </c>
@@ -1582,7 +1579,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:19">
       <c r="A6">
         <v>1015105</v>
       </c>
@@ -1641,7 +1638,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:19">
       <c r="A7">
         <v>1015107</v>
       </c>
@@ -1700,7 +1697,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:19">
       <c r="A8">
         <v>1015179</v>
       </c>
@@ -1759,7 +1756,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:19">
       <c r="A9">
         <v>1015477</v>
       </c>
@@ -1818,7 +1815,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:19">
       <c r="A10">
         <v>1015752</v>
       </c>
@@ -1877,7 +1874,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:19">
       <c r="A11">
         <v>1015778</v>
       </c>
@@ -1936,7 +1933,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:19">
       <c r="A12">
         <v>1017402</v>
       </c>
@@ -1995,7 +1992,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:19">
       <c r="A13">
         <v>1045997</v>
       </c>
@@ -2054,7 +2051,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:19">
       <c r="A14">
         <v>1046386</v>
       </c>
@@ -2113,7 +2110,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:19">
       <c r="A15">
         <v>1046386</v>
       </c>
@@ -2172,7 +2169,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:19">
       <c r="A16">
         <v>1046386</v>
       </c>
@@ -2231,7 +2228,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:19">
       <c r="A17">
         <v>1046386</v>
       </c>
@@ -2290,7 +2287,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:19">
       <c r="A18">
         <v>1046386</v>
       </c>
@@ -2349,7 +2346,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:19">
       <c r="A19">
         <v>1046386</v>
       </c>
@@ -2408,7 +2405,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:19">
       <c r="A20">
         <v>1046386</v>
       </c>
@@ -2467,7 +2464,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="21" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:19">
       <c r="A21">
         <v>1046386</v>
       </c>
@@ -2526,7 +2523,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="22" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:19">
       <c r="A22">
         <v>1046386</v>
       </c>
@@ -2585,7 +2582,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="23" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:19">
       <c r="A23">
         <v>1046508</v>
       </c>
@@ -2644,7 +2641,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="24" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:19">
       <c r="A24">
         <v>1046508</v>
       </c>
@@ -2703,7 +2700,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="25" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:19">
       <c r="A25">
         <v>1046508</v>
       </c>
@@ -2762,7 +2759,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="26" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:19">
       <c r="A26">
         <v>1046566</v>
       </c>
@@ -2821,7 +2818,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="27" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:19">
       <c r="A27">
         <v>1046566</v>
       </c>
@@ -2880,7 +2877,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="28" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:19">
       <c r="A28">
         <v>1046612</v>
       </c>
@@ -2939,7 +2936,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="29" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:19">
       <c r="A29">
         <v>1046612</v>
       </c>
@@ -2998,7 +2995,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="30" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:19">
       <c r="A30">
         <v>1046612</v>
       </c>
@@ -3057,7 +3054,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="31" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:19">
       <c r="A31">
         <v>1083463</v>
       </c>
@@ -3116,7 +3113,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="32" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:19">
       <c r="A32">
         <v>1083470</v>
       </c>
@@ -3175,7 +3172,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="33" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:19">
       <c r="A33">
         <v>1083476</v>
       </c>
@@ -3234,7 +3231,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="34" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:19">
       <c r="A34">
         <v>1083696</v>
       </c>
@@ -3293,7 +3290,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="35" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:19">
       <c r="A35">
         <v>1083696</v>
       </c>
@@ -3352,7 +3349,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="36" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:19">
       <c r="A36">
         <v>1083696</v>
       </c>
@@ -3411,7 +3408,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="37" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:19">
       <c r="A37">
         <v>1083696</v>
       </c>
@@ -3470,7 +3467,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="38" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:19">
       <c r="A38">
         <v>1083696</v>
       </c>
@@ -3529,7 +3526,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="39" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:19">
       <c r="A39">
         <v>1083696</v>
       </c>
@@ -3588,7 +3585,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="40" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:19">
       <c r="A40">
         <v>1083696</v>
       </c>
@@ -3647,7 +3644,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="41" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:19">
       <c r="A41">
         <v>1086853</v>
       </c>
@@ -3706,7 +3703,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="42" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:19">
       <c r="A42">
         <v>1086853</v>
       </c>
@@ -3765,7 +3762,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="43" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:19">
       <c r="A43">
         <v>1086853</v>
       </c>
@@ -3824,7 +3821,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="44" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:19">
       <c r="A44">
         <v>1086853</v>
       </c>
@@ -3883,7 +3880,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="45" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:19">
       <c r="A45">
         <v>1086853</v>
       </c>
@@ -3942,7 +3939,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="46" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:19">
       <c r="A46">
         <v>1086853</v>
       </c>
@@ -4001,7 +3998,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="47" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:19">
       <c r="A47">
         <v>1086853</v>
       </c>
@@ -4060,7 +4057,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="48" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:19">
       <c r="A48">
         <v>1086859</v>
       </c>
@@ -4119,7 +4116,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="49" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:19">
       <c r="A49">
         <v>1086859</v>
       </c>
@@ -4178,7 +4175,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="50" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:19">
       <c r="A50">
         <v>1086859</v>
       </c>
@@ -4237,7 +4234,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="51" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:19">
       <c r="A51">
         <v>1086859</v>
       </c>
@@ -4296,7 +4293,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="52" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:19">
       <c r="A52">
         <v>1086859</v>
       </c>
@@ -4355,7 +4352,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="53" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:19">
       <c r="A53">
         <v>1086859</v>
       </c>
@@ -4414,7 +4411,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="54" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:19">
       <c r="A54">
         <v>1086859</v>
       </c>
@@ -4473,7 +4470,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="55" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:19">
       <c r="A55">
         <v>1086865</v>
       </c>
@@ -4532,7 +4529,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="56" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:19">
       <c r="A56">
         <v>1086865</v>
       </c>
@@ -4591,7 +4588,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="57" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:19">
       <c r="A57">
         <v>1086865</v>
       </c>
@@ -4650,7 +4647,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="58" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:19">
       <c r="A58">
         <v>1086865</v>
       </c>
@@ -4709,7 +4706,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="59" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:19">
       <c r="A59">
         <v>1086865</v>
       </c>
@@ -4768,7 +4765,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="60" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:19">
       <c r="A60">
         <v>1086865</v>
       </c>
@@ -4827,7 +4824,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="61" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:19">
       <c r="A61">
         <v>1086865</v>
       </c>
@@ -4886,7 +4883,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="62" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:19">
       <c r="A62">
         <v>1086871</v>
       </c>
@@ -4945,7 +4942,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="63" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:19">
       <c r="A63">
         <v>1086871</v>
       </c>
@@ -5004,7 +5001,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="64" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:19">
       <c r="A64">
         <v>1086871</v>
       </c>
@@ -5063,7 +5060,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="65" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:19">
       <c r="A65">
         <v>1086871</v>
       </c>
@@ -5122,7 +5119,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="66" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:19">
       <c r="A66">
         <v>1086871</v>
       </c>
@@ -5181,7 +5178,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="67" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:19">
       <c r="A67">
         <v>1086871</v>
       </c>
@@ -5240,7 +5237,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="68" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:19">
       <c r="A68">
         <v>1086871</v>
       </c>
@@ -5299,7 +5296,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="69" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:19">
       <c r="A69">
         <v>1086915</v>
       </c>
@@ -5358,7 +5355,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="70" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:19">
       <c r="A70">
         <v>1086928</v>
       </c>
@@ -5417,7 +5414,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="71" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:19">
       <c r="A71">
         <v>1086998</v>
       </c>
@@ -5476,7 +5473,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="72" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:19">
       <c r="A72">
         <v>1087006</v>
       </c>
@@ -5535,7 +5532,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="73" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:19">
       <c r="A73">
         <v>1087017</v>
       </c>
@@ -5594,7 +5591,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="74" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:19">
       <c r="A74">
         <v>1087021</v>
       </c>
@@ -5653,7 +5650,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="75" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:19">
       <c r="A75">
         <v>1087025</v>
       </c>
@@ -5712,7 +5709,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="76" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:19">
       <c r="A76">
         <v>1087032</v>
       </c>
@@ -5771,7 +5768,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="77" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:19">
       <c r="A77">
         <v>1087039</v>
       </c>
@@ -5830,7 +5827,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="78" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:19">
       <c r="A78">
         <v>1087048</v>
       </c>
@@ -5889,7 +5886,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="79" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:19">
       <c r="A79">
         <v>1087695</v>
       </c>
@@ -5948,7 +5945,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="80" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:19">
       <c r="A80">
         <v>1087697</v>
       </c>
@@ -6007,7 +6004,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="81" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:19">
       <c r="A81">
         <v>1087699</v>
       </c>
@@ -6066,7 +6063,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="82" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:19">
       <c r="A82">
         <v>1087700</v>
       </c>
@@ -6125,7 +6122,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="83" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:19">
       <c r="A83">
         <v>1087700</v>
       </c>
@@ -6184,7 +6181,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="84" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:19">
       <c r="A84">
         <v>1087703</v>
       </c>
@@ -6243,7 +6240,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="85" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:19">
       <c r="A85">
         <v>1087720</v>
       </c>
@@ -6302,7 +6299,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="86" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:19">
       <c r="A86">
         <v>1087722</v>
       </c>
@@ -6361,7 +6358,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="87" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:19">
       <c r="A87">
         <v>1087724</v>
       </c>
@@ -6420,7 +6417,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="88" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:19">
       <c r="A88">
         <v>1087724</v>
       </c>
@@ -6479,7 +6476,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="89" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:19">
       <c r="A89">
         <v>1087739</v>
       </c>
@@ -6538,7 +6535,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="90" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:19">
       <c r="A90">
         <v>1087748</v>
       </c>
@@ -6597,7 +6594,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="91" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:19">
       <c r="A91">
         <v>1087752</v>
       </c>
@@ -6656,7 +6653,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="92" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:19">
       <c r="A92">
         <v>1087757</v>
       </c>
@@ -6715,7 +6712,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="93" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:19">
       <c r="A93">
         <v>1087763</v>
       </c>
@@ -6774,7 +6771,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="94" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:19">
       <c r="A94">
         <v>1087770</v>
       </c>
@@ -6833,7 +6830,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="95" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:19">
       <c r="A95">
         <v>1087784</v>
       </c>
@@ -6892,7 +6889,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="96" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:19">
       <c r="A96">
         <v>1087792</v>
       </c>
@@ -6951,7 +6948,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="97" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:19">
       <c r="A97">
         <v>1087800</v>
       </c>
@@ -7010,7 +7007,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="98" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:19">
       <c r="A98">
         <v>1087800</v>
       </c>
@@ -7069,7 +7066,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="99" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:19">
       <c r="A99">
         <v>1087806</v>
       </c>
@@ -7128,7 +7125,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="100" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:19">
       <c r="A100">
         <v>1087814</v>
       </c>
@@ -7187,7 +7184,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="101" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:19">
       <c r="A101">
         <v>1087823</v>
       </c>
@@ -7246,7 +7243,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="102" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:19">
       <c r="A102">
         <v>1087854</v>
       </c>
@@ -7305,7 +7302,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="103" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:19">
       <c r="A103">
         <v>1087854</v>
       </c>
@@ -7364,7 +7361,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="104" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:19">
       <c r="A104">
         <v>1087856</v>
       </c>
@@ -7423,7 +7420,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="105" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:19">
       <c r="A105">
         <v>1087874</v>
       </c>
@@ -7482,7 +7479,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="106" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:19">
       <c r="A106">
         <v>1087880</v>
       </c>
@@ -7541,7 +7538,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="107" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:19">
       <c r="A107">
         <v>1093542</v>
       </c>
@@ -7600,7 +7597,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="108" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:19">
       <c r="A108">
         <v>1093546</v>
       </c>
@@ -7659,7 +7656,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="109" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:19">
       <c r="A109">
         <v>1093555</v>
       </c>
@@ -7718,7 +7715,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="110" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:19">
       <c r="A110">
         <v>1093580</v>
       </c>
@@ -7777,7 +7774,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="111" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:19">
       <c r="A111">
         <v>1093594</v>
       </c>
@@ -7836,7 +7833,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="112" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:19">
       <c r="A112">
         <v>1093659</v>
       </c>
@@ -7895,7 +7892,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="113" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:19">
       <c r="A113">
         <v>1093668</v>
       </c>
@@ -7954,7 +7951,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="114" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:19">
       <c r="A114">
         <v>1093671</v>
       </c>
@@ -8013,7 +8010,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="115" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:19">
       <c r="A115">
         <v>1093756</v>
       </c>
@@ -8072,7 +8069,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="116" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:19">
       <c r="A116">
         <v>1093786</v>
       </c>
@@ -8131,7 +8128,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="117" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:19">
       <c r="A117">
         <v>1093786</v>
       </c>
@@ -8190,7 +8187,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="118" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:19">
       <c r="A118">
         <v>1093899</v>
       </c>
@@ -8249,7 +8246,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="119" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:19">
       <c r="A119">
         <v>1093899</v>
       </c>
@@ -8308,7 +8305,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="120" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:19">
       <c r="A120">
         <v>1094006</v>
       </c>
@@ -8367,7 +8364,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="121" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:19">
       <c r="A121">
         <v>1094006</v>
       </c>
@@ -8426,7 +8423,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="122" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:19">
       <c r="A122">
         <v>1094012</v>
       </c>
@@ -8485,7 +8482,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="123" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:19">
       <c r="A123">
         <v>1094012</v>
       </c>
@@ -8544,7 +8541,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="124" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:19">
       <c r="A124">
         <v>1094020</v>
       </c>
@@ -8603,7 +8600,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="125" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:19">
       <c r="A125">
         <v>1094048</v>
       </c>
@@ -8662,7 +8659,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="126" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:19">
       <c r="A126">
         <v>1094051</v>
       </c>
@@ -8721,7 +8718,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="127" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:19">
       <c r="A127">
         <v>1094060</v>
       </c>
@@ -8780,7 +8777,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="128" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:19">
       <c r="A128">
         <v>1094060</v>
       </c>
@@ -8839,7 +8836,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="129" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:19">
       <c r="A129">
         <v>1094131</v>
       </c>
@@ -8898,7 +8895,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="130" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:19">
       <c r="A130">
         <v>1094529</v>
       </c>
@@ -8957,7 +8954,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="131" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:19">
       <c r="A131">
         <v>1094534</v>
       </c>
@@ -9016,7 +9013,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="132" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:19">
       <c r="A132">
         <v>1094538</v>
       </c>
@@ -9075,7 +9072,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="133" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:19">
       <c r="A133">
         <v>1094774</v>
       </c>
@@ -9134,7 +9131,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="134" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:19">
       <c r="A134">
         <v>1094846</v>
       </c>
@@ -9193,7 +9190,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="135" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:19">
       <c r="A135">
         <v>1094887</v>
       </c>
@@ -9252,7 +9249,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="136" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:19">
       <c r="A136">
         <v>1094918</v>
       </c>
@@ -9311,7 +9308,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="137" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:19">
       <c r="A137">
         <v>1094933</v>
       </c>
@@ -9370,7 +9367,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="138" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:19">
       <c r="A138">
         <v>1094942</v>
       </c>
@@ -9429,7 +9426,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="139" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:19">
       <c r="A139">
         <v>1094942</v>
       </c>
@@ -9488,7 +9485,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="140" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:19">
       <c r="A140">
         <v>1095014</v>
       </c>
@@ -9547,7 +9544,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="141" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:19">
       <c r="A141">
         <v>1095035</v>
       </c>
@@ -9606,7 +9603,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="142" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:19">
       <c r="A142">
         <v>1095041</v>
       </c>
@@ -9665,7 +9662,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="143" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:19">
       <c r="A143">
         <v>1095077</v>
       </c>
@@ -9724,7 +9721,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="144" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:19">
       <c r="A144">
         <v>1095082</v>
       </c>
@@ -9783,7 +9780,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="145" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:19">
       <c r="A145">
         <v>1095094</v>
       </c>
@@ -9842,7 +9839,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="146" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:19">
       <c r="A146">
         <v>1095152</v>
       </c>
@@ -9901,7 +9898,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="147" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:19">
       <c r="A147">
         <v>1095165</v>
       </c>
@@ -9960,7 +9957,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="148" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:19">
       <c r="A148">
         <v>1095179</v>
       </c>
@@ -10019,7 +10016,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="149" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:19">
       <c r="A149">
         <v>1095201</v>
       </c>
@@ -10078,7 +10075,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="150" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:19">
       <c r="A150">
         <v>1095226</v>
       </c>
@@ -10137,7 +10134,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="151" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:19">
       <c r="A151">
         <v>1095257</v>
       </c>
@@ -10196,7 +10193,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="152" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:19">
       <c r="A152">
         <v>1095257</v>
       </c>
@@ -10255,7 +10252,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="153" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:19">
       <c r="A153">
         <v>1095257</v>
       </c>
@@ -10314,7 +10311,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="154" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:19">
       <c r="A154">
         <v>1095257</v>
       </c>
@@ -10373,7 +10370,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="155" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:19">
       <c r="A155">
         <v>1095257</v>
       </c>
@@ -10432,7 +10429,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="156" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:19">
       <c r="A156">
         <v>1095257</v>
       </c>
@@ -10491,7 +10488,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="157" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:19">
       <c r="A157">
         <v>1095257</v>
       </c>
@@ -10550,7 +10547,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="158" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:19">
       <c r="A158">
         <v>1095269</v>
       </c>
@@ -10609,7 +10606,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="159" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:19">
       <c r="A159">
         <v>1095269</v>
       </c>
@@ -10668,7 +10665,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="160" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:19">
       <c r="A160">
         <v>1095269</v>
       </c>
@@ -10727,7 +10724,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="161" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:19">
       <c r="A161">
         <v>1095269</v>
       </c>
@@ -10786,7 +10783,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="162" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:19">
       <c r="A162">
         <v>1095269</v>
       </c>
@@ -10845,7 +10842,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="163" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:19">
       <c r="A163">
         <v>1095269</v>
       </c>
@@ -10904,7 +10901,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="164" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:19">
       <c r="A164">
         <v>1095269</v>
       </c>
@@ -10963,7 +10960,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="165" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:19">
       <c r="A165">
         <v>1095275</v>
       </c>
@@ -11022,7 +11019,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="166" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:19">
       <c r="A166">
         <v>1095275</v>
       </c>
@@ -11081,7 +11078,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="167" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:19">
       <c r="A167">
         <v>1095275</v>
       </c>
@@ -11140,7 +11137,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="168" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:19">
       <c r="A168">
         <v>1095275</v>
       </c>
@@ -11199,7 +11196,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="169" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:19">
       <c r="A169">
         <v>1095275</v>
       </c>
@@ -11258,7 +11255,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="170" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:19">
       <c r="A170">
         <v>1095275</v>
       </c>
@@ -11317,7 +11314,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="171" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:19">
       <c r="A171">
         <v>1095275</v>
       </c>
@@ -11376,7 +11373,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="172" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:19">
       <c r="A172">
         <v>1095464</v>
       </c>
@@ -11435,7 +11432,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="173" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:19">
       <c r="A173">
         <v>1095482</v>
       </c>
@@ -11494,7 +11491,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="174" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:19">
       <c r="A174">
         <v>1095505</v>
       </c>
@@ -11553,7 +11550,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="175" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:19">
       <c r="A175">
         <v>1095510</v>
       </c>
@@ -11612,7 +11609,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="176" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:19">
       <c r="A176">
         <v>1095534</v>
       </c>
@@ -11671,7 +11668,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="177" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:19">
       <c r="A177">
         <v>1095535</v>
       </c>
@@ -11730,7 +11727,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="178" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:19">
       <c r="A178">
         <v>1095562</v>
       </c>
@@ -11789,7 +11786,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="179" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:19">
       <c r="A179">
         <v>1095572</v>
       </c>
@@ -11848,7 +11845,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="180" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:19">
       <c r="A180">
         <v>1095576</v>
       </c>
@@ -11907,7 +11904,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="181" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:19">
       <c r="A181">
         <v>1095578</v>
       </c>
@@ -11966,7 +11963,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="182" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:19">
       <c r="A182">
         <v>1095584</v>
       </c>
@@ -12025,7 +12022,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="183" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:19">
       <c r="A183">
         <v>1095588</v>
       </c>
@@ -12084,7 +12081,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="184" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:19">
       <c r="A184">
         <v>1095591</v>
       </c>
@@ -12143,7 +12140,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="185" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:19">
       <c r="A185">
         <v>1095616</v>
       </c>
@@ -12202,7 +12199,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="186" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:19">
       <c r="A186">
         <v>1095628</v>
       </c>
@@ -12261,7 +12258,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="187" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:19">
       <c r="A187">
         <v>1095628</v>
       </c>
@@ -12320,7 +12317,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="188" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:19">
       <c r="A188">
         <v>1095628</v>
       </c>
@@ -12379,7 +12376,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="189" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:19">
       <c r="A189">
         <v>1095633</v>
       </c>
@@ -12438,7 +12435,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="190" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:19">
       <c r="A190">
         <v>1095635</v>
       </c>
@@ -12497,7 +12494,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="191" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:19">
       <c r="A191">
         <v>1095638</v>
       </c>
@@ -12556,7 +12553,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="192" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:19">
       <c r="A192">
         <v>1095648</v>
       </c>
@@ -12615,7 +12612,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="193" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:19">
       <c r="A193">
         <v>1095651</v>
       </c>
@@ -12674,7 +12671,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="194" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:19">
       <c r="A194">
         <v>1095652</v>
       </c>
@@ -12733,7 +12730,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="195" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:19">
       <c r="A195">
         <v>1095661</v>
       </c>
@@ -12792,7 +12789,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="196" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:19">
       <c r="A196">
         <v>1095668</v>
       </c>
@@ -12851,7 +12848,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="197" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:19">
       <c r="A197">
         <v>1095679</v>
       </c>
@@ -12910,7 +12907,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="198" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:19">
       <c r="A198">
         <v>1095690</v>
       </c>
@@ -12969,7 +12966,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="199" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:19">
       <c r="A199">
         <v>1095691</v>
       </c>
@@ -13028,7 +13025,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="200" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:19">
       <c r="A200">
         <v>1095701</v>
       </c>
@@ -13087,7 +13084,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="201" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:19">
       <c r="A201">
         <v>1095709</v>
       </c>
@@ -13146,7 +13143,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="202" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:19">
       <c r="A202">
         <v>1095719</v>
       </c>
@@ -13205,7 +13202,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="203" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:19">
       <c r="A203">
         <v>1095725</v>
       </c>
@@ -13264,7 +13261,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="204" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:19">
       <c r="A204">
         <v>1095726</v>
       </c>
@@ -13323,7 +13320,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="205" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:19">
       <c r="A205">
         <v>1095743</v>
       </c>
@@ -13382,7 +13379,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="206" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:19">
       <c r="A206">
         <v>1095745</v>
       </c>
@@ -13441,7 +13438,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="207" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:19">
       <c r="A207">
         <v>1095757</v>
       </c>
@@ -13500,7 +13497,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="208" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:19">
       <c r="A208">
         <v>1095764</v>
       </c>
@@ -13559,7 +13556,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="209" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:19">
       <c r="A209">
         <v>1095764</v>
       </c>
@@ -13618,7 +13615,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="210" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:19">
       <c r="A210">
         <v>1095774</v>
       </c>
@@ -13677,7 +13674,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="211" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:19">
       <c r="A211">
         <v>1095778</v>
       </c>
@@ -13736,7 +13733,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="212" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:19">
       <c r="A212">
         <v>1095781</v>
       </c>
@@ -13795,7 +13792,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="213" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:19">
       <c r="A213">
         <v>1095787</v>
       </c>
@@ -13854,7 +13851,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="214" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:19">
       <c r="A214">
         <v>1095793</v>
       </c>
@@ -13913,7 +13910,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="215" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:19">
       <c r="A215">
         <v>1095800</v>
       </c>
@@ -13972,7 +13969,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="216" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:19">
       <c r="A216">
         <v>1095809</v>
       </c>
@@ -14031,7 +14028,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="217" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:19">
       <c r="A217">
         <v>1095811</v>
       </c>
@@ -14090,7 +14087,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="218" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:19">
       <c r="A218">
         <v>1095814</v>
       </c>
@@ -14149,7 +14146,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="219" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:19">
       <c r="A219">
         <v>1095821</v>
       </c>
@@ -14208,7 +14205,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="220" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:19">
       <c r="A220">
         <v>1095824</v>
       </c>
@@ -14267,7 +14264,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="221" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:19">
       <c r="A221">
         <v>1095825</v>
       </c>
@@ -14326,7 +14323,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="222" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:19">
       <c r="A222">
         <v>1095830</v>
       </c>
@@ -14385,7 +14382,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="223" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:19">
       <c r="A223">
         <v>1095846</v>
       </c>
@@ -14444,7 +14441,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="224" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:19">
       <c r="A224">
         <v>1095852</v>
       </c>
@@ -14503,7 +14500,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="225" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:19">
       <c r="A225">
         <v>1095858</v>
       </c>
@@ -14562,7 +14559,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="226" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:19">
       <c r="A226">
         <v>1095860</v>
       </c>
@@ -14621,7 +14618,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="227" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:19">
       <c r="A227">
         <v>1095870</v>
       </c>
@@ -14680,7 +14677,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="228" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:19">
       <c r="A228">
         <v>1095874</v>
       </c>
@@ -14739,7 +14736,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="229" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:19">
       <c r="A229">
         <v>1095875</v>
       </c>
@@ -14798,7 +14795,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="230" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:19">
       <c r="A230">
         <v>1095880</v>
       </c>
@@ -14857,7 +14854,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="231" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:19">
       <c r="A231">
         <v>1095891</v>
       </c>
@@ -14916,7 +14913,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="232" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:19">
       <c r="A232">
         <v>1095892</v>
       </c>
@@ -14975,7 +14972,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="233" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:19">
       <c r="A233">
         <v>1095896</v>
       </c>
@@ -15034,7 +15031,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="234" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:19">
       <c r="A234">
         <v>1095908</v>
       </c>
@@ -15093,7 +15090,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="235" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:19">
       <c r="A235">
         <v>1095919</v>
       </c>
@@ -15152,7 +15149,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="236" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:19">
       <c r="A236">
         <v>1095919</v>
       </c>
@@ -15211,7 +15208,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="237" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:19">
       <c r="A237">
         <v>1095919</v>
       </c>
@@ -15270,7 +15267,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="238" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:19">
       <c r="A238">
         <v>1095926</v>
       </c>
@@ -15329,7 +15326,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="239" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:19">
       <c r="A239">
         <v>1095942</v>
       </c>
@@ -15388,7 +15385,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="240" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:19">
       <c r="A240">
         <v>1095949</v>
       </c>
@@ -15447,7 +15444,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="241" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:19">
       <c r="A241">
         <v>1095949</v>
       </c>
@@ -15506,7 +15503,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="242" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:19">
       <c r="A242">
         <v>1095949</v>
       </c>
@@ -15565,7 +15562,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="243" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:19">
       <c r="A243">
         <v>1095949</v>
       </c>
@@ -15624,7 +15621,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="244" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:19">
       <c r="A244">
         <v>1095950</v>
       </c>
@@ -15683,7 +15680,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="245" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:19">
       <c r="A245">
         <v>1095960</v>
       </c>
@@ -15742,7 +15739,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="246" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:19">
       <c r="A246">
         <v>1095973</v>
       </c>
@@ -15801,7 +15798,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="247" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:19">
       <c r="A247">
         <v>1095976</v>
       </c>
@@ -15860,7 +15857,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="248" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:19">
       <c r="A248">
         <v>1095976</v>
       </c>
@@ -15919,7 +15916,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="249" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:19">
       <c r="A249">
         <v>1095985</v>
       </c>
@@ -15978,7 +15975,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="250" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:19">
       <c r="A250">
         <v>1095990</v>
       </c>
@@ -16037,7 +16034,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="251" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:19">
       <c r="A251">
         <v>1096008</v>
       </c>
@@ -16096,7 +16093,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="252" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:19">
       <c r="A252">
         <v>1096021</v>
       </c>
@@ -16155,7 +16152,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="253" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:19">
       <c r="A253">
         <v>1096053</v>
       </c>
@@ -16214,7 +16211,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="254" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:19">
       <c r="A254">
         <v>1096054</v>
       </c>
@@ -16273,7 +16270,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="255" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:19">
       <c r="A255">
         <v>1096054</v>
       </c>
@@ -16332,7 +16329,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="256" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:19">
       <c r="A256">
         <v>1096063</v>
       </c>
@@ -16391,7 +16388,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="257" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:19">
       <c r="A257">
         <v>1096063</v>
       </c>
@@ -16450,7 +16447,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="258" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:19">
       <c r="A258">
         <v>1096072</v>
       </c>
@@ -16509,7 +16506,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="259" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:19">
       <c r="A259">
         <v>1096072</v>
       </c>
@@ -16568,7 +16565,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="260" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:19">
       <c r="A260">
         <v>1096081</v>
       </c>
@@ -16627,7 +16624,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="261" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:19">
       <c r="A261">
         <v>1096081</v>
       </c>
@@ -16686,7 +16683,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="262" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:19">
       <c r="A262">
         <v>1096084</v>
       </c>
@@ -16745,7 +16742,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="263" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:19">
       <c r="A263">
         <v>1096089</v>
       </c>
@@ -16804,7 +16801,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="264" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:19">
       <c r="A264">
         <v>1096115</v>
       </c>
@@ -16863,7 +16860,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="265" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:19">
       <c r="A265">
         <v>1096117</v>
       </c>
@@ -16922,7 +16919,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="266" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:19">
       <c r="A266">
         <v>1096130</v>
       </c>
@@ -16981,7 +16978,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="267" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:19">
       <c r="A267">
         <v>1096138</v>
       </c>
@@ -17040,7 +17037,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="268" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:19">
       <c r="A268">
         <v>1096143</v>
       </c>
@@ -17099,7 +17096,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="269" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:19">
       <c r="A269">
         <v>1096143</v>
       </c>
@@ -17158,7 +17155,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="270" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:19">
       <c r="A270">
         <v>1096143</v>
       </c>
@@ -17217,7 +17214,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="271" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:19">
       <c r="A271">
         <v>1096147</v>
       </c>
@@ -17276,7 +17273,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="272" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:19">
       <c r="A272">
         <v>1096165</v>
       </c>
@@ -17335,7 +17332,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="273" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:19">
       <c r="A273">
         <v>1096165</v>
       </c>
@@ -17394,7 +17391,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="274" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:19">
       <c r="A274">
         <v>1096165</v>
       </c>
@@ -17453,7 +17450,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="275" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:19">
       <c r="A275">
         <v>1096213</v>
       </c>
@@ -17512,7 +17509,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="276" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:19">
       <c r="A276">
         <v>1096234</v>
       </c>
@@ -17571,7 +17568,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="277" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:19">
       <c r="A277">
         <v>1096427</v>
       </c>
@@ -17630,7 +17627,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="278" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:19">
       <c r="A278">
         <v>1096565</v>
       </c>
@@ -17689,7 +17686,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="279" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:19">
       <c r="A279">
         <v>1096571</v>
       </c>
@@ -17748,7 +17745,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="280" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:19">
       <c r="A280">
         <v>1096636</v>
       </c>
@@ -17807,7 +17804,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="281" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:19">
       <c r="A281">
         <v>1097087</v>
       </c>
@@ -17866,7 +17863,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="282" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:19">
       <c r="A282">
         <v>1097093</v>
       </c>
@@ -17925,7 +17922,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="283" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:19">
       <c r="A283">
         <v>1097097</v>
       </c>
@@ -17984,7 +17981,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="284" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="284" spans="1:19">
       <c r="A284">
         <v>1097114</v>
       </c>
@@ -18043,7 +18040,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="285" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="285" spans="1:19">
       <c r="A285">
         <v>1097114</v>
       </c>
@@ -18102,7 +18099,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="286" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="286" spans="1:19">
       <c r="A286">
         <v>1097114</v>
       </c>
@@ -18161,7 +18158,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="287" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="287" spans="1:19">
       <c r="A287">
         <v>1097114</v>
       </c>
@@ -18220,7 +18217,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="288" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="288" spans="1:19">
       <c r="A288">
         <v>1097114</v>
       </c>
@@ -18279,7 +18276,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="289" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="289" spans="1:19">
       <c r="A289">
         <v>1097114</v>
       </c>
@@ -18338,7 +18335,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="290" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="290" spans="1:19">
       <c r="A290">
         <v>1097132</v>
       </c>
@@ -18397,7 +18394,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="291" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="291" spans="1:19">
       <c r="A291">
         <v>1097132</v>
       </c>
@@ -18456,7 +18453,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="292" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="292" spans="1:19">
       <c r="A292">
         <v>1097132</v>
       </c>
@@ -18515,7 +18512,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="293" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="293" spans="1:19">
       <c r="A293">
         <v>1097132</v>
       </c>
@@ -18574,7 +18571,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="294" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="294" spans="1:19">
       <c r="A294">
         <v>1097132</v>
       </c>
@@ -18633,7 +18630,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="295" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="295" spans="1:19">
       <c r="A295">
         <v>1097171</v>
       </c>
@@ -18692,7 +18689,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="296" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="296" spans="1:19">
       <c r="A296">
         <v>1097325</v>
       </c>
@@ -18751,7 +18748,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="297" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="297" spans="1:19">
       <c r="A297">
         <v>1097425</v>
       </c>
@@ -18765,7 +18762,7 @@
         <v>21</v>
       </c>
       <c r="E297">
-        <v>49.990001678467003</v>
+        <v>49.990001678467</v>
       </c>
       <c r="F297" t="s">
         <v>19</v>
@@ -18810,7 +18807,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="298" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="298" spans="1:19">
       <c r="A298">
         <v>1097450</v>
       </c>
@@ -18869,7 +18866,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="299" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="299" spans="1:19">
       <c r="A299">
         <v>1097521</v>
       </c>
@@ -18928,7 +18925,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="300" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="300" spans="1:19">
       <c r="A300">
         <v>1097546</v>
       </c>
@@ -18987,7 +18984,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="301" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="301" spans="1:19">
       <c r="A301">
         <v>1097546</v>
       </c>
@@ -19046,7 +19043,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="302" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="302" spans="1:19">
       <c r="A302">
         <v>1097551</v>
       </c>
@@ -19105,7 +19102,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="303" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="303" spans="1:19">
       <c r="A303">
         <v>1097582</v>
       </c>
@@ -19164,7 +19161,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="304" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="304" spans="1:19">
       <c r="A304">
         <v>1097591</v>
       </c>
@@ -19223,7 +19220,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="305" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="305" spans="1:19">
       <c r="A305">
         <v>1097655</v>
       </c>
@@ -19282,7 +19279,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="306" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="306" spans="1:19">
       <c r="A306">
         <v>1097716</v>
       </c>
@@ -19341,7 +19338,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="307" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="307" spans="1:19">
       <c r="A307">
         <v>1097716</v>
       </c>
@@ -19400,7 +19397,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="308" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="308" spans="1:19">
       <c r="A308">
         <v>1097716</v>
       </c>
@@ -19459,7 +19456,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="309" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="309" spans="1:19">
       <c r="A309">
         <v>1097809</v>
       </c>
@@ -19518,7 +19515,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="310" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="310" spans="1:19">
       <c r="A310">
         <v>1098514</v>
       </c>
@@ -19577,7 +19574,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="311" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="311" spans="1:19">
       <c r="A311">
         <v>1098541</v>
       </c>
@@ -19636,7 +19633,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="312" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="312" spans="1:19">
       <c r="A312">
         <v>1098594</v>
       </c>
@@ -19695,7 +19692,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="313" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="313" spans="1:19">
       <c r="A313">
         <v>1098635</v>
       </c>
@@ -19709,7 +19706,7 @@
         <v>21</v>
       </c>
       <c r="E313">
-        <v>9.9899997711181996</v>
+        <v>9.9899997711182</v>
       </c>
       <c r="F313" t="s">
         <v>19</v>
@@ -19754,7 +19751,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="314" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="314" spans="1:19">
       <c r="A314">
         <v>1098636</v>
       </c>
@@ -19813,7 +19810,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="315" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="315" spans="1:19">
       <c r="A315">
         <v>1098636</v>
       </c>
@@ -19872,7 +19869,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="316" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="316" spans="1:19">
       <c r="A316">
         <v>1098647</v>
       </c>
@@ -19931,7 +19928,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="317" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="317" spans="1:19">
       <c r="A317">
         <v>1098676</v>
       </c>
@@ -19990,7 +19987,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="318" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="318" spans="1:19">
       <c r="A318">
         <v>1098713</v>
       </c>
@@ -20049,7 +20046,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="319" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="319" spans="1:19">
       <c r="A319">
         <v>1098726</v>
       </c>
@@ -20108,7 +20105,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="320" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="320" spans="1:19">
       <c r="A320">
         <v>1098744</v>
       </c>
@@ -20167,7 +20164,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="321" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="321" spans="1:19">
       <c r="A321">
         <v>1098773</v>
       </c>
@@ -20226,7 +20223,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="322" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="322" spans="1:19">
       <c r="A322">
         <v>1098842</v>
       </c>
@@ -20285,7 +20282,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="323" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="323" spans="1:19">
       <c r="A323">
         <v>1098846</v>
       </c>
@@ -20344,7 +20341,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="324" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="324" spans="1:19">
       <c r="A324">
         <v>1098886</v>
       </c>
@@ -20403,7 +20400,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="325" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="325" spans="1:19">
       <c r="A325">
         <v>1099695</v>
       </c>
@@ -20462,7 +20459,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="326" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="326" spans="1:19">
       <c r="A326">
         <v>1099715</v>
       </c>
@@ -20521,7 +20518,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="327" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="327" spans="1:19">
       <c r="A327">
         <v>1099759</v>
       </c>
@@ -20580,7 +20577,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="328" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="328" spans="1:19">
       <c r="A328">
         <v>1099767</v>
       </c>
@@ -20639,7 +20636,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="329" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="329" spans="1:19">
       <c r="A329">
         <v>1099777</v>
       </c>
@@ -20698,7 +20695,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="330" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="330" spans="1:19">
       <c r="A330">
         <v>1099778</v>
       </c>
@@ -20757,7 +20754,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="331" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="331" spans="1:19">
       <c r="A331">
         <v>1099802</v>
       </c>
@@ -20816,7 +20813,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="332" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="332" spans="1:19">
       <c r="A332">
         <v>1099815</v>
       </c>
@@ -20875,7 +20872,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="333" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="333" spans="1:19">
       <c r="A333">
         <v>1100416</v>
       </c>
@@ -20934,7 +20931,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="334" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="334" spans="1:19">
       <c r="A334">
         <v>1100819</v>
       </c>
@@ -20993,7 +20990,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="335" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="335" spans="1:19">
       <c r="A335">
         <v>1100819</v>
       </c>
@@ -21052,7 +21049,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="336" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="336" spans="1:19">
       <c r="A336">
         <v>1100820</v>
       </c>
@@ -21111,7 +21108,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="337" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="337" spans="1:19">
       <c r="A337">
         <v>1100821</v>
       </c>
@@ -21170,7 +21167,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="338" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="338" spans="1:19">
       <c r="A338">
         <v>1100824</v>
       </c>
@@ -21229,7 +21226,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="339" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="339" spans="1:19">
       <c r="A339">
         <v>1100824</v>
       </c>
@@ -21288,7 +21285,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="340" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="340" spans="1:19">
       <c r="A340">
         <v>1100886</v>
       </c>
@@ -21347,7 +21344,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="341" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="341" spans="1:19">
       <c r="A341">
         <v>1101512</v>
       </c>
@@ -21406,7 +21403,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="342" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="342" spans="1:19">
       <c r="A342">
         <v>1101672</v>
       </c>
@@ -21465,7 +21462,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="343" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="343" spans="1:19">
       <c r="A343">
         <v>1103027</v>
       </c>
@@ -21524,7 +21521,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="344" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="344" spans="1:19">
       <c r="A344">
         <v>1103031</v>
       </c>
@@ -21583,7 +21580,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="345" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="345" spans="1:19">
       <c r="A345">
         <v>1103108</v>
       </c>
@@ -21642,7 +21639,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="346" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="346" spans="1:19">
       <c r="A346">
         <v>1103126</v>
       </c>
@@ -21701,7 +21698,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="347" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="347" spans="1:19">
       <c r="A347">
         <v>1103139</v>
       </c>
@@ -21760,7 +21757,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="348" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="348" spans="1:19">
       <c r="A348">
         <v>1103147</v>
       </c>
@@ -21819,7 +21816,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="349" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="349" spans="1:19">
       <c r="A349">
         <v>1103156</v>
       </c>
@@ -21878,7 +21875,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="350" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="350" spans="1:19">
       <c r="A350">
         <v>1103161</v>
       </c>
@@ -21937,7 +21934,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="351" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="351" spans="1:19">
       <c r="A351">
         <v>1103168</v>
       </c>
@@ -21996,7 +21993,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="352" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="352" spans="1:19">
       <c r="A352">
         <v>1103186</v>
       </c>
@@ -22055,7 +22052,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="353" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="353" spans="1:19">
       <c r="A353">
         <v>1103186</v>
       </c>
@@ -22114,7 +22111,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="354" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="354" spans="1:19">
       <c r="A354">
         <v>1103192</v>
       </c>
@@ -22173,7 +22170,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="355" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="355" spans="1:19">
       <c r="A355">
         <v>1103197</v>
       </c>
@@ -22232,7 +22229,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="356" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="356" spans="1:19">
       <c r="A356">
         <v>1103294</v>
       </c>
@@ -22291,7 +22288,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="357" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="357" spans="1:19">
       <c r="A357">
         <v>1103294</v>
       </c>
@@ -22350,7 +22347,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="358" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="358" spans="1:19">
       <c r="A358">
         <v>1103297</v>
       </c>
@@ -22409,7 +22406,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="359" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="359" spans="1:19">
       <c r="A359">
         <v>1103297</v>
       </c>
@@ -22468,7 +22465,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="360" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="360" spans="1:19">
       <c r="A360">
         <v>1103297</v>
       </c>
@@ -22527,7 +22524,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="361" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="361" spans="1:19">
       <c r="A361">
         <v>1103297</v>
       </c>
@@ -22586,7 +22583,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="362" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="362" spans="1:19">
       <c r="A362">
         <v>1103345</v>
       </c>
@@ -22645,7 +22642,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="363" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="363" spans="1:19">
       <c r="A363">
         <v>1103381</v>
       </c>
@@ -22704,7 +22701,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="364" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="364" spans="1:19">
       <c r="A364">
         <v>1103381</v>
       </c>
@@ -22763,7 +22760,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="365" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="365" spans="1:19">
       <c r="A365">
         <v>1103386</v>
       </c>
@@ -22822,7 +22819,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="366" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="366" spans="1:19">
       <c r="A366">
         <v>1103387</v>
       </c>
@@ -22881,7 +22878,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="367" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="367" spans="1:19">
       <c r="A367">
         <v>1103387</v>
       </c>
@@ -22940,7 +22937,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="368" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="368" spans="1:19">
       <c r="A368">
         <v>1103387</v>
       </c>
@@ -22999,7 +22996,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="369" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="369" spans="1:19">
       <c r="A369">
         <v>1103387</v>
       </c>
@@ -23058,7 +23055,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="370" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="370" spans="1:19">
       <c r="A370">
         <v>1103388</v>
       </c>
@@ -23117,7 +23114,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="371" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="371" spans="1:19">
       <c r="A371">
         <v>1103388</v>
       </c>
@@ -23176,7 +23173,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="372" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="372" spans="1:19">
       <c r="A372">
         <v>1103388</v>
       </c>
@@ -23235,7 +23232,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="373" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="373" spans="1:19">
       <c r="A373">
         <v>1103388</v>
       </c>
@@ -23294,7 +23291,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="374" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="374" spans="1:19">
       <c r="A374">
         <v>1103394</v>
       </c>
@@ -23353,7 +23350,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="375" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="375" spans="1:19">
       <c r="A375">
         <v>1103412</v>
       </c>
@@ -23412,7 +23409,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="376" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="376" spans="1:19">
       <c r="A376">
         <v>1103436</v>
       </c>
@@ -23471,7 +23468,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="377" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="377" spans="1:19">
       <c r="A377">
         <v>1103495</v>
       </c>
@@ -23530,7 +23527,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="378" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="378" spans="1:19">
       <c r="A378">
         <v>1103845</v>
       </c>
@@ -23589,7 +23586,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="379" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="379" spans="1:19">
       <c r="A379">
         <v>1104405</v>
       </c>
@@ -23648,7 +23645,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="380" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="380" spans="1:19">
       <c r="A380">
         <v>1104405</v>
       </c>
@@ -23707,7 +23704,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="381" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="381" spans="1:19">
       <c r="A381">
         <v>1104408</v>
       </c>
@@ -23766,7 +23763,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="382" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="382" spans="1:19">
       <c r="A382">
         <v>1104408</v>
       </c>
@@ -23825,7 +23822,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="383" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="383" spans="1:19">
       <c r="A383">
         <v>1105361</v>
       </c>
@@ -23884,7 +23881,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="384" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="384" spans="1:19">
       <c r="A384">
         <v>1105367</v>
       </c>
@@ -23943,7 +23940,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="385" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="385" spans="1:19">
       <c r="A385">
         <v>1105372</v>
       </c>
@@ -24002,7 +23999,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="386" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="386" spans="1:19">
       <c r="A386">
         <v>1105376</v>
       </c>
@@ -24061,7 +24058,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="387" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="387" spans="1:19">
       <c r="A387">
         <v>1107240</v>
       </c>
@@ -24120,7 +24117,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="388" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="388" spans="1:19">
       <c r="A388">
         <v>1107240</v>
       </c>
@@ -24179,7 +24176,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="389" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="389" spans="1:19">
       <c r="A389">
         <v>1107240</v>
       </c>
@@ -24238,7 +24235,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="390" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="390" spans="1:19">
       <c r="A390">
         <v>1107261</v>
       </c>
@@ -24297,7 +24294,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="391" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="391" spans="1:19">
       <c r="A391">
         <v>1107261</v>
       </c>
@@ -24356,7 +24353,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="392" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="392" spans="1:19">
       <c r="A392">
         <v>1107261</v>
       </c>
@@ -24415,7 +24412,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="393" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="393" spans="1:19">
       <c r="A393">
         <v>1108775</v>
       </c>
@@ -24474,7 +24471,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="394" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="394" spans="1:19">
       <c r="A394">
         <v>1112923</v>
       </c>
@@ -24533,7 +24530,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="395" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="395" spans="1:19">
       <c r="A395">
         <v>1113717</v>
       </c>
@@ -24592,7 +24589,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="396" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="396" spans="1:19">
       <c r="A396">
         <v>1115949</v>
       </c>
@@ -24651,7 +24648,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="397" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="397" spans="1:19">
       <c r="A397">
         <v>1115949</v>
       </c>
@@ -24710,7 +24707,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="398" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="398" spans="1:19">
       <c r="A398">
         <v>1115949</v>
       </c>
@@ -24769,7 +24766,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="399" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="399" spans="1:19">
       <c r="A399">
         <v>1119669</v>
       </c>
@@ -24828,7 +24825,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="400" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="400" spans="1:19">
       <c r="A400">
         <v>1122417</v>
       </c>
@@ -24887,7 +24884,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="401" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="401" spans="1:19">
       <c r="A401">
         <v>1122986</v>
       </c>
@@ -24946,7 +24943,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="402" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="402" spans="1:19">
       <c r="A402">
         <v>1122990</v>
       </c>
@@ -25005,7 +25002,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="403" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="403" spans="1:19">
       <c r="A403">
         <v>1122994</v>
       </c>
@@ -25064,7 +25061,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="404" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="404" spans="1:19">
       <c r="A404">
         <v>1122998</v>
       </c>
@@ -25123,7 +25120,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="405" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="405" spans="1:19">
       <c r="A405">
         <v>1127005</v>
       </c>
@@ -25182,7 +25179,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="406" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="406" spans="1:19">
       <c r="A406">
         <v>1127037</v>
       </c>
@@ -25241,7 +25238,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="407" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="407" spans="1:19">
       <c r="A407">
         <v>1135668</v>
       </c>
@@ -25300,7 +25297,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="408" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="408" spans="1:19">
       <c r="A408">
         <v>1135675</v>
       </c>
@@ -25359,7 +25356,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="409" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="409" spans="1:19">
       <c r="A409">
         <v>1135679</v>
       </c>
@@ -25418,7 +25415,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="410" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="410" spans="1:19">
       <c r="A410">
         <v>1135679</v>
       </c>
@@ -25477,7 +25474,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="411" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="411" spans="1:19">
       <c r="A411">
         <v>1135685</v>
       </c>
@@ -25536,7 +25533,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="412" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="412" spans="1:19">
       <c r="A412">
         <v>1135690</v>
       </c>
@@ -25595,7 +25592,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="413" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="413" spans="1:19">
       <c r="A413">
         <v>1135699</v>
       </c>
@@ -25654,7 +25651,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="414" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="414" spans="1:19">
       <c r="A414">
         <v>1135706</v>
       </c>
@@ -25713,7 +25710,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="415" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="415" spans="1:19">
       <c r="A415">
         <v>1135710</v>
       </c>
@@ -25772,7 +25769,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="416" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="416" spans="1:19">
       <c r="A416">
         <v>1225107</v>
       </c>
@@ -25831,7 +25828,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="417" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="417" spans="1:19">
       <c r="A417">
         <v>1229486</v>
       </c>
@@ -25890,7 +25887,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="418" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="418" spans="1:19">
       <c r="A418">
         <v>1229486</v>
       </c>
@@ -25949,7 +25946,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="419" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="419" spans="1:19">
       <c r="A419">
         <v>1229486</v>
       </c>
@@ -26008,7 +26005,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="420" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="420" spans="1:19">
       <c r="A420">
         <v>1229486</v>
       </c>
@@ -26067,7 +26064,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="421" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="421" spans="1:19">
       <c r="A421">
         <v>1229486</v>
       </c>
@@ -26126,7 +26123,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="422" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="422" spans="1:19">
       <c r="A422">
         <v>1229486</v>
       </c>
@@ -26185,7 +26182,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="423" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="423" spans="1:19">
       <c r="A423">
         <v>1229486</v>
       </c>
@@ -26244,7 +26241,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="424" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="424" spans="1:19">
       <c r="A424">
         <v>1229486</v>
       </c>
@@ -26303,7 +26300,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="425" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="425" spans="1:19">
       <c r="A425">
         <v>1229486</v>
       </c>
@@ -26362,7 +26359,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="426" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="426" spans="1:19">
       <c r="A426">
         <v>1229486</v>
       </c>
@@ -26421,7 +26418,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="427" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="427" spans="1:19">
       <c r="A427">
         <v>1229486</v>
       </c>
@@ -26480,7 +26477,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="428" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="428" spans="1:19">
       <c r="A428">
         <v>1229486</v>
       </c>
@@ -26539,7 +26536,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="429" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="429" spans="1:19">
       <c r="A429">
         <v>1229486</v>
       </c>
@@ -26598,7 +26595,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="430" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="430" spans="1:19">
       <c r="A430">
         <v>1229486</v>
       </c>
@@ -26657,7 +26654,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="431" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="431" spans="1:19">
       <c r="A431">
         <v>1229486</v>
       </c>
@@ -26716,7 +26713,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="432" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="432" spans="1:19">
       <c r="A432">
         <v>1229486</v>
       </c>
@@ -26775,7 +26772,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="433" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="433" spans="1:19">
       <c r="A433">
         <v>1229486</v>
       </c>
@@ -26834,7 +26831,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="434" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="434" spans="1:19">
       <c r="A434">
         <v>1229486</v>
       </c>
@@ -26893,7 +26890,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="435" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="435" spans="1:19">
       <c r="A435">
         <v>1229486</v>
       </c>
@@ -26952,7 +26949,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="436" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="436" spans="1:19">
       <c r="A436">
         <v>1229486</v>
       </c>
@@ -27011,7 +27008,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="437" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="437" spans="1:19">
       <c r="A437">
         <v>1229486</v>
       </c>
@@ -27070,7 +27067,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="438" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="438" spans="1:19">
       <c r="A438">
         <v>1229486</v>
       </c>
@@ -27129,7 +27126,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="439" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="439" spans="1:19">
       <c r="A439">
         <v>1229486</v>
       </c>
@@ -27188,7 +27185,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="440" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="440" spans="1:19">
       <c r="A440">
         <v>1229486</v>
       </c>
@@ -27247,7 +27244,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="441" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="441" spans="1:19">
       <c r="A441">
         <v>1229486</v>
       </c>
@@ -27306,7 +27303,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="442" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="442" spans="1:19">
       <c r="A442">
         <v>1229486</v>
       </c>
@@ -27365,7 +27362,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="443" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="443" spans="1:19">
       <c r="A443">
         <v>1229486</v>
       </c>
@@ -27424,7 +27421,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="444" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="444" spans="1:19">
       <c r="A444">
         <v>1229486</v>
       </c>
@@ -27483,7 +27480,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="445" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="445" spans="1:19">
       <c r="A445">
         <v>1229486</v>
       </c>
@@ -27542,7 +27539,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="446" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="446" spans="1:19">
       <c r="A446">
         <v>1229486</v>
       </c>
@@ -27601,7 +27598,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="447" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="447" spans="1:19">
       <c r="A447">
         <v>1229486</v>
       </c>
@@ -27660,7 +27657,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="448" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="448" spans="1:19">
       <c r="A448">
         <v>1229486</v>
       </c>
@@ -27719,7 +27716,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="449" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="449" spans="1:19">
       <c r="A449">
         <v>1229486</v>
       </c>
@@ -27778,7 +27775,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="450" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="450" spans="1:19">
       <c r="A450">
         <v>1229486</v>
       </c>
@@ -27837,7 +27834,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="451" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="451" spans="1:19">
       <c r="A451">
         <v>1229486</v>
       </c>
@@ -27896,7 +27893,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="452" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="452" spans="1:19">
       <c r="A452">
         <v>1229486</v>
       </c>
@@ -27956,6 +27953,17 @@
       </c>
     </row>
   </sheetData>
+  <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
+  <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
+    <oddHeader/>
+    <oddFooter/>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+  <tableParts count="0"/>
 </worksheet>
 </file>
</xml_diff>